<commit_message>
create 2024vs2025 or 2025vs2026 diff code
</commit_message>
<xml_diff>
--- a/mvp_comparison_2025_vs_2026.xlsx
+++ b/mvp_comparison_2025_vs_2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\playground\mvpspdier2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\playground\mvp-year-diff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3B53D3D-19F2-47C5-AC8B-37591390487B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5072846-59A4-4B68-A313-DEF1EBB12695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -594,10 +594,10 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -905,7 +905,9 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="10.109375" style="3" customWidth="1"/>
+    <col min="2" max="3" width="11.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.77734375" style="3" customWidth="1"/>
+    <col min="5" max="5" width="12.109375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>